<commit_message>
Add initiative options tab to unmapped review workbook
</commit_message>
<xml_diff>
--- a/data/unmapped_review_first_pass.xlsx
+++ b/data/unmapped_review_first_pass.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="review_queue" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="quick_pick" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="initiative_options" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +33,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="4">
@@ -66,10 +71,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -20606,4 +20612,320 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Initiative Selection Options</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Initiative Classification</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Matrix Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tokenized Securities / RWA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Assets</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Traditional financial assets represented on blockchain rails.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DLT / Blockchain Infrastructure</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Core ledger and platform infrastructure enabling digital asset use cases.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Crypto / Digital Assets</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Assets</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Native digital asset activity and crypto market infrastructure.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Payment Infrastructure</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Payment rail execution including domestic and cross-border flows.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Stablecoins &amp; Deposit Tokens</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Fiat-referenced digital money instruments and related workflows.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CBDC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Public Money</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Central bank digital currency pilots, policy, and implementations.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DeFi</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Decentralized Markets</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Decentralized protocol-based financial activity.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Digital Asset Strategy</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Enterprise strategic posture, governance, and capability planning.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Interoperability &amp; Standards</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Standards and mechanisms connecting systems and ledgers.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Settlement Infrastructure</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Market Structure</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Clearing, settlement finality, collateral, and post-trade rails.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Regulatory / Compliance</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Policy</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Regulatory frameworks, supervision, and compliance controls.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cross-Border Payments</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Alias mapped to Payment Infrastructure for matrix consistency.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>